<commit_message>
Adding loops to ODK file
</commit_message>
<xml_diff>
--- a/dictionary/variables_master.xlsx
+++ b/dictionary/variables_master.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eafit-my.sharepoint.com/personal/rszapatav_eafit_edu_co/Documents/CIAT/Metodología Evaluaciones/surveyProcessingMethodology/dictionary/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="195" documentId="8_{4C1B0862-69B3-42BC-8750-06EDE6596D4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86EBA8C0-3889-4C1E-BFE3-132486A16A78}"/>
+  <xr:revisionPtr revIDLastSave="286" documentId="8_{4C1B0862-69B3-42BC-8750-06EDE6596D4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6207DBD-6E4A-4466-9FDF-B443C4302FD9}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-4725" windowWidth="29040" windowHeight="15720" xr2:uid="{D5E2868F-FAC0-444C-BFCE-6871238D4C9E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{D5E2868F-FAC0-444C-BFCE-6871238D4C9E}"/>
   </bookViews>
   <sheets>
-    <sheet name="variables_master" sheetId="1" r:id="rId1"/>
+    <sheet name="variables_master2" sheetId="1" r:id="rId1"/>
+    <sheet name="variables_master" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="164">
   <si>
     <t>variable_name</t>
   </si>
@@ -477,13 +478,61 @@
   </si>
   <si>
     <t>catuai:Catuaí­|caturra:Caturra|bourbon:Bourbon|geisha:Geisha|lempira:Lempira|ihcafe90:IHCAFE 90|pacas:Pacas|other:Otra</t>
+  </si>
+  <si>
+    <t>surv_required</t>
+  </si>
+  <si>
+    <t>surv_relevant</t>
+  </si>
+  <si>
+    <t>surv_constraint</t>
+  </si>
+  <si>
+    <t>surv_constraint_message</t>
+  </si>
+  <si>
+    <t>surv_choices</t>
+  </si>
+  <si>
+    <t>surv_type</t>
+  </si>
+  <si>
+    <t>surv_hint</t>
+  </si>
+  <si>
+    <t>surv_choice_filter</t>
+  </si>
+  <si>
+    <t>surv_repeat_count</t>
+  </si>
+  <si>
+    <t>surv_calculation</t>
+  </si>
+  <si>
+    <t>surv_calculation_output</t>
+  </si>
+  <si>
+    <t>surv_calculation_include</t>
+  </si>
+  <si>
+    <t>subtopic</t>
+  </si>
+  <si>
+    <t>plot_loop</t>
+  </si>
+  <si>
+    <t>${area_total_farm_raw}&gt;0</t>
+  </si>
+  <si>
+    <t>${farm_count}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -618,8 +667,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -799,6 +854,12 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -960,9 +1021,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="13" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1342,7 +1404,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.140625" style="1"/>
+    <col min="14" max="23" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.25">
@@ -1373,7 +1435,7 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
       <c r="K1" t="s">
@@ -1435,7 +1497,7 @@
       <c r="G2">
         <v>1</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2">
         <v>1</v>
       </c>
       <c r="K2">
@@ -1482,7 +1544,7 @@
       <c r="I3" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3">
         <v>0</v>
       </c>
       <c r="L3" t="s">
@@ -1541,7 +1603,7 @@
       <c r="G4">
         <v>1</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4">
         <v>0</v>
       </c>
       <c r="L4" t="s">
@@ -1597,7 +1659,7 @@
       <c r="I5" t="s">
         <v>64</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5">
         <v>0</v>
       </c>
       <c r="L5" t="s">
@@ -1659,7 +1721,7 @@
       <c r="I6" t="s">
         <v>68</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6">
         <v>0</v>
       </c>
       <c r="L6" t="s">
@@ -1718,7 +1780,7 @@
       <c r="G7">
         <v>1</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7">
         <v>0</v>
       </c>
       <c r="L7" t="s">
@@ -1774,7 +1836,7 @@
       <c r="I8" t="s">
         <v>41</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8">
         <v>0</v>
       </c>
       <c r="L8" t="s">
@@ -1836,7 +1898,7 @@
       <c r="I9" t="s">
         <v>46</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9">
         <v>0</v>
       </c>
       <c r="K9" t="s">
@@ -1898,7 +1960,7 @@
       <c r="G10">
         <v>1</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10">
         <v>0</v>
       </c>
       <c r="L10" t="s">
@@ -1945,7 +2007,7 @@
       <c r="I11" t="s">
         <v>46</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11">
         <v>0</v>
       </c>
       <c r="K11" t="s">
@@ -2007,7 +2069,7 @@
       <c r="G12">
         <v>1</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12">
         <v>0</v>
       </c>
       <c r="L12" t="s">
@@ -2063,7 +2125,7 @@
       <c r="I13" t="s">
         <v>79</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13">
         <v>0</v>
       </c>
       <c r="K13" t="s">
@@ -2125,7 +2187,7 @@
       <c r="G14">
         <v>1</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14">
         <v>0</v>
       </c>
       <c r="L14" t="s">
@@ -2172,7 +2234,7 @@
       <c r="I15" t="s">
         <v>91</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15">
         <v>0</v>
       </c>
       <c r="L15" t="s">
@@ -2231,7 +2293,7 @@
       <c r="G16">
         <v>1</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16">
         <v>0</v>
       </c>
       <c r="L16" t="s">
@@ -2284,7 +2346,7 @@
       <c r="G17">
         <v>1</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17">
         <v>0</v>
       </c>
       <c r="L17" t="s">
@@ -2340,7 +2402,7 @@
       <c r="I18" t="s">
         <v>100</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18">
         <v>0</v>
       </c>
       <c r="L18" t="s">
@@ -2399,7 +2461,7 @@
       <c r="G19">
         <v>1</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19">
         <v>0</v>
       </c>
       <c r="L19" t="s">
@@ -2455,7 +2517,7 @@
       <c r="I20" t="s">
         <v>107</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20">
         <v>0</v>
       </c>
       <c r="L20" t="s">
@@ -2514,7 +2576,7 @@
       <c r="G21">
         <v>1</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21">
         <v>0</v>
       </c>
       <c r="L21" t="s">
@@ -2570,7 +2632,7 @@
       <c r="I22" t="s">
         <v>117</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22">
         <v>0</v>
       </c>
       <c r="L22" t="s">
@@ -2623,7 +2685,7 @@
       <c r="I23" t="s">
         <v>122</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23">
         <v>0</v>
       </c>
       <c r="L23" t="s">
@@ -2676,7 +2738,7 @@
       <c r="I24" t="s">
         <v>127</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24">
         <v>0</v>
       </c>
       <c r="L24" t="s">
@@ -2729,7 +2791,7 @@
       <c r="G25">
         <v>1</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25">
         <v>0</v>
       </c>
       <c r="L25" t="s">
@@ -2748,6 +2810,1539 @@
         <v>0</v>
       </c>
       <c r="U25">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B98D0170-56BF-40AD-B5DE-47C0DB191985}">
+  <dimension ref="A1:AC25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
+    <col min="7" max="7" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="15.7109375" customWidth="1"/>
+    <col min="10" max="10" width="19" customWidth="1"/>
+    <col min="11" max="11" width="14.42578125" customWidth="1"/>
+    <col min="12" max="12" width="14.140625" customWidth="1"/>
+    <col min="13" max="13" width="16.42578125" customWidth="1"/>
+    <col min="14" max="14" width="25.140625" customWidth="1"/>
+    <col min="15" max="15" width="21.85546875" customWidth="1"/>
+    <col min="16" max="16" width="17.140625" customWidth="1"/>
+    <col min="17" max="17" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="21.85546875" customWidth="1"/>
+    <col min="20" max="29" width="9.140625" hidden="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:29" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="X2">
+        <v>0</v>
+      </c>
+      <c r="Y2">
+        <v>0</v>
+      </c>
+      <c r="AB2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3" t="s">
+        <v>31</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="M3" t="s">
+        <v>32</v>
+      </c>
+      <c r="N3" t="s">
+        <v>33</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>28</v>
+      </c>
+      <c r="T3">
+        <v>1</v>
+      </c>
+      <c r="U3">
+        <v>18</v>
+      </c>
+      <c r="V3">
+        <v>100</v>
+      </c>
+      <c r="W3">
+        <v>3</v>
+      </c>
+      <c r="X3">
+        <v>1</v>
+      </c>
+      <c r="Y3">
+        <v>1</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB3">
+        <v>3</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4" t="s">
+        <v>60</v>
+      </c>
+      <c r="I4" t="s">
+        <v>130</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>57</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+      <c r="X4">
+        <v>1</v>
+      </c>
+      <c r="Y4">
+        <v>1</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB4">
+        <v>3</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E5" t="s">
+        <v>62</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5" t="s">
+        <v>31</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="M5" t="s">
+        <v>63</v>
+      </c>
+      <c r="N5" t="s">
+        <v>64</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>61</v>
+      </c>
+      <c r="T5">
+        <v>1</v>
+      </c>
+      <c r="U5">
+        <v>1</v>
+      </c>
+      <c r="V5">
+        <v>20</v>
+      </c>
+      <c r="W5">
+        <v>3</v>
+      </c>
+      <c r="X5">
+        <v>1</v>
+      </c>
+      <c r="Y5">
+        <v>1</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB5">
+        <v>3</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>65</v>
+      </c>
+      <c r="D6" t="s">
+        <v>134</v>
+      </c>
+      <c r="E6" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6" t="s">
+        <v>31</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="M6" t="s">
+        <v>67</v>
+      </c>
+      <c r="N6" t="s">
+        <v>68</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>65</v>
+      </c>
+      <c r="T6">
+        <v>1</v>
+      </c>
+      <c r="U6">
+        <v>0</v>
+      </c>
+      <c r="V6">
+        <v>70</v>
+      </c>
+      <c r="W6">
+        <v>3</v>
+      </c>
+      <c r="X6">
+        <v>1</v>
+      </c>
+      <c r="Y6">
+        <v>1</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB6">
+        <v>3</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D7" t="s">
+        <v>135</v>
+      </c>
+      <c r="E7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7" t="s">
+        <v>60</v>
+      </c>
+      <c r="I7" t="s">
+        <v>145</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>69</v>
+      </c>
+      <c r="T7">
+        <v>0</v>
+      </c>
+      <c r="W7">
+        <v>0</v>
+      </c>
+      <c r="X7">
+        <v>1</v>
+      </c>
+      <c r="Y7">
+        <v>1</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB7">
+        <v>3</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8" t="s">
+        <v>31</v>
+      </c>
+      <c r="K8">
+        <v>1</v>
+      </c>
+      <c r="M8" t="s">
+        <v>40</v>
+      </c>
+      <c r="N8" t="s">
+        <v>41</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>37</v>
+      </c>
+      <c r="T8">
+        <v>1</v>
+      </c>
+      <c r="U8">
+        <v>1</v>
+      </c>
+      <c r="V8">
+        <v>10</v>
+      </c>
+      <c r="W8">
+        <v>2</v>
+      </c>
+      <c r="X8">
+        <v>1</v>
+      </c>
+      <c r="Y8">
+        <v>1</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB8">
+        <v>3</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" t="s">
+        <v>161</v>
+      </c>
+      <c r="C9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" t="s">
+        <v>56</v>
+      </c>
+      <c r="E9" t="s">
+        <v>51</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9" t="s">
+        <v>44</v>
+      </c>
+      <c r="K9">
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
+        <v>45</v>
+      </c>
+      <c r="N9" t="s">
+        <v>46</v>
+      </c>
+      <c r="O9">
+        <v>1</v>
+      </c>
+      <c r="P9" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>53</v>
+      </c>
+      <c r="R9" t="s">
+        <v>163</v>
+      </c>
+      <c r="T9">
+        <v>1</v>
+      </c>
+      <c r="U9">
+        <v>0</v>
+      </c>
+      <c r="V9">
+        <v>200</v>
+      </c>
+      <c r="W9">
+        <v>3</v>
+      </c>
+      <c r="X9">
+        <v>1</v>
+      </c>
+      <c r="Y9">
+        <v>1</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB9">
+        <v>3</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" t="s">
+        <v>161</v>
+      </c>
+      <c r="C10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D10" t="s">
+        <v>136</v>
+      </c>
+      <c r="E10" t="s">
+        <v>72</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10" t="s">
+        <v>60</v>
+      </c>
+      <c r="I10" t="s">
+        <v>146</v>
+      </c>
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>71</v>
+      </c>
+      <c r="R10" t="s">
+        <v>163</v>
+      </c>
+      <c r="T10">
+        <v>0</v>
+      </c>
+      <c r="W10">
+        <v>0</v>
+      </c>
+      <c r="X10">
+        <v>0</v>
+      </c>
+      <c r="AA10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" t="s">
+        <v>161</v>
+      </c>
+      <c r="C11" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" t="s">
+        <v>55</v>
+      </c>
+      <c r="E11" t="s">
+        <v>43</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11" t="s">
+        <v>44</v>
+      </c>
+      <c r="K11">
+        <v>1</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="M11" t="s">
+        <v>45</v>
+      </c>
+      <c r="N11" t="s">
+        <v>46</v>
+      </c>
+      <c r="O11">
+        <v>1</v>
+      </c>
+      <c r="P11" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>48</v>
+      </c>
+      <c r="R11" t="s">
+        <v>163</v>
+      </c>
+      <c r="T11">
+        <v>1</v>
+      </c>
+      <c r="U11">
+        <v>0</v>
+      </c>
+      <c r="V11">
+        <v>50</v>
+      </c>
+      <c r="W11">
+        <v>3</v>
+      </c>
+      <c r="X11">
+        <v>1</v>
+      </c>
+      <c r="Y11">
+        <v>1</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB11">
+        <v>2</v>
+      </c>
+      <c r="AC11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C12" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" t="s">
+        <v>137</v>
+      </c>
+      <c r="E12" t="s">
+        <v>74</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12" t="s">
+        <v>60</v>
+      </c>
+      <c r="I12" t="s">
+        <v>147</v>
+      </c>
+      <c r="K12">
+        <v>1</v>
+      </c>
+      <c r="O12">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>73</v>
+      </c>
+      <c r="T12">
+        <v>0</v>
+      </c>
+      <c r="W12">
+        <v>0</v>
+      </c>
+      <c r="X12">
+        <v>1</v>
+      </c>
+      <c r="Y12">
+        <v>1</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB12">
+        <v>3</v>
+      </c>
+      <c r="AC12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>75</v>
+      </c>
+      <c r="B13" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" t="s">
+        <v>76</v>
+      </c>
+      <c r="D13" t="s">
+        <v>138</v>
+      </c>
+      <c r="E13" t="s">
+        <v>77</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13" t="s">
+        <v>44</v>
+      </c>
+      <c r="K13">
+        <v>1</v>
+      </c>
+      <c r="M13" t="s">
+        <v>78</v>
+      </c>
+      <c r="N13" t="s">
+        <v>79</v>
+      </c>
+      <c r="O13">
+        <v>1</v>
+      </c>
+      <c r="P13" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>81</v>
+      </c>
+      <c r="T13">
+        <v>1</v>
+      </c>
+      <c r="U13">
+        <v>0</v>
+      </c>
+      <c r="V13">
+        <v>10000</v>
+      </c>
+      <c r="W13">
+        <v>3</v>
+      </c>
+      <c r="X13">
+        <v>1</v>
+      </c>
+      <c r="Y13">
+        <v>1</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB13">
+        <v>1</v>
+      </c>
+      <c r="AC13" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="14" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" t="s">
+        <v>83</v>
+      </c>
+      <c r="D14" t="s">
+        <v>85</v>
+      </c>
+      <c r="E14" t="s">
+        <v>84</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14" t="s">
+        <v>60</v>
+      </c>
+      <c r="I14" t="s">
+        <v>131</v>
+      </c>
+      <c r="K14">
+        <v>1</v>
+      </c>
+      <c r="O14">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>83</v>
+      </c>
+      <c r="T14">
+        <v>0</v>
+      </c>
+      <c r="W14">
+        <v>0</v>
+      </c>
+      <c r="X14">
+        <v>0</v>
+      </c>
+      <c r="AA14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>89</v>
+      </c>
+      <c r="B15" t="s">
+        <v>89</v>
+      </c>
+      <c r="C15" t="s">
+        <v>86</v>
+      </c>
+      <c r="D15" t="s">
+        <v>88</v>
+      </c>
+      <c r="E15" t="s">
+        <v>87</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K15">
+        <v>1</v>
+      </c>
+      <c r="M15" t="s">
+        <v>90</v>
+      </c>
+      <c r="N15" t="s">
+        <v>91</v>
+      </c>
+      <c r="O15">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>92</v>
+      </c>
+      <c r="T15">
+        <v>1</v>
+      </c>
+      <c r="U15">
+        <v>0</v>
+      </c>
+      <c r="V15">
+        <v>1000</v>
+      </c>
+      <c r="W15">
+        <v>3</v>
+      </c>
+      <c r="X15">
+        <v>1</v>
+      </c>
+      <c r="Y15">
+        <v>1</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB15">
+        <v>2</v>
+      </c>
+      <c r="AC15" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="16" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>89</v>
+      </c>
+      <c r="B16" t="s">
+        <v>89</v>
+      </c>
+      <c r="C16" t="s">
+        <v>93</v>
+      </c>
+      <c r="D16" t="s">
+        <v>139</v>
+      </c>
+      <c r="E16" t="s">
+        <v>94</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16" t="s">
+        <v>60</v>
+      </c>
+      <c r="I16" t="s">
+        <v>132</v>
+      </c>
+      <c r="K16">
+        <v>1</v>
+      </c>
+      <c r="O16">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>93</v>
+      </c>
+      <c r="T16">
+        <v>0</v>
+      </c>
+      <c r="W16">
+        <v>0</v>
+      </c>
+      <c r="X16">
+        <v>1</v>
+      </c>
+      <c r="Y16">
+        <v>1</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB16">
+        <v>2</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="17" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" t="s">
+        <v>97</v>
+      </c>
+      <c r="C17" t="s">
+        <v>95</v>
+      </c>
+      <c r="D17" t="s">
+        <v>140</v>
+      </c>
+      <c r="E17" t="s">
+        <v>96</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17" t="s">
+        <v>60</v>
+      </c>
+      <c r="I17" t="s">
+        <v>132</v>
+      </c>
+      <c r="K17">
+        <v>1</v>
+      </c>
+      <c r="O17">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>95</v>
+      </c>
+      <c r="T17">
+        <v>0</v>
+      </c>
+      <c r="W17">
+        <v>0</v>
+      </c>
+      <c r="X17">
+        <v>1</v>
+      </c>
+      <c r="Y17">
+        <v>1</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB17">
+        <v>2</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>97</v>
+      </c>
+      <c r="B18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C18" t="s">
+        <v>98</v>
+      </c>
+      <c r="D18" t="s">
+        <v>141</v>
+      </c>
+      <c r="E18" t="s">
+        <v>99</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18" t="s">
+        <v>44</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="M18" t="s">
+        <v>78</v>
+      </c>
+      <c r="N18" t="s">
+        <v>100</v>
+      </c>
+      <c r="O18">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>98</v>
+      </c>
+      <c r="T18">
+        <v>1</v>
+      </c>
+      <c r="U18">
+        <v>0</v>
+      </c>
+      <c r="V18">
+        <v>50000</v>
+      </c>
+      <c r="W18">
+        <v>3</v>
+      </c>
+      <c r="X18">
+        <v>1</v>
+      </c>
+      <c r="Y18">
+        <v>1</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB18">
+        <v>2</v>
+      </c>
+      <c r="AC18" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>103</v>
+      </c>
+      <c r="B19" t="s">
+        <v>103</v>
+      </c>
+      <c r="C19" t="s">
+        <v>101</v>
+      </c>
+      <c r="D19" t="s">
+        <v>142</v>
+      </c>
+      <c r="E19" t="s">
+        <v>102</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19" t="s">
+        <v>60</v>
+      </c>
+      <c r="I19" t="s">
+        <v>132</v>
+      </c>
+      <c r="K19">
+        <v>1</v>
+      </c>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>101</v>
+      </c>
+      <c r="T19">
+        <v>0</v>
+      </c>
+      <c r="W19">
+        <v>0</v>
+      </c>
+      <c r="X19">
+        <v>1</v>
+      </c>
+      <c r="Y19">
+        <v>1</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB19">
+        <v>2</v>
+      </c>
+      <c r="AC19" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>103</v>
+      </c>
+      <c r="B20" t="s">
+        <v>103</v>
+      </c>
+      <c r="C20" t="s">
+        <v>104</v>
+      </c>
+      <c r="D20" t="s">
+        <v>106</v>
+      </c>
+      <c r="E20" t="s">
+        <v>105</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20" t="s">
+        <v>44</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="M20" t="s">
+        <v>78</v>
+      </c>
+      <c r="N20" t="s">
+        <v>107</v>
+      </c>
+      <c r="O20">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>104</v>
+      </c>
+      <c r="T20">
+        <v>1</v>
+      </c>
+      <c r="U20">
+        <v>0</v>
+      </c>
+      <c r="V20">
+        <v>5000</v>
+      </c>
+      <c r="W20">
+        <v>3</v>
+      </c>
+      <c r="X20">
+        <v>1</v>
+      </c>
+      <c r="Y20">
+        <v>1</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB20">
+        <v>3</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>111</v>
+      </c>
+      <c r="B21" t="s">
+        <v>111</v>
+      </c>
+      <c r="C21" t="s">
+        <v>108</v>
+      </c>
+      <c r="D21" t="s">
+        <v>110</v>
+      </c>
+      <c r="E21" t="s">
+        <v>109</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+      <c r="G21" t="s">
+        <v>60</v>
+      </c>
+      <c r="I21" t="s">
+        <v>132</v>
+      </c>
+      <c r="K21">
+        <v>1</v>
+      </c>
+      <c r="O21">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>108</v>
+      </c>
+      <c r="T21">
+        <v>0</v>
+      </c>
+      <c r="W21">
+        <v>0</v>
+      </c>
+      <c r="X21">
+        <v>1</v>
+      </c>
+      <c r="Y21">
+        <v>1</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB21">
+        <v>2</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="22" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>115</v>
+      </c>
+      <c r="B22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C22" t="s">
+        <v>112</v>
+      </c>
+      <c r="D22" t="s">
+        <v>114</v>
+      </c>
+      <c r="E22" t="s">
+        <v>113</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22" t="s">
+        <v>44</v>
+      </c>
+      <c r="K22">
+        <v>0</v>
+      </c>
+      <c r="M22" t="s">
+        <v>116</v>
+      </c>
+      <c r="N22" t="s">
+        <v>117</v>
+      </c>
+      <c r="O22">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>112</v>
+      </c>
+      <c r="T22">
+        <v>1</v>
+      </c>
+      <c r="U22">
+        <v>-90</v>
+      </c>
+      <c r="V22">
+        <v>90</v>
+      </c>
+      <c r="W22">
+        <v>0</v>
+      </c>
+      <c r="X22">
+        <v>0</v>
+      </c>
+      <c r="AA22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>115</v>
+      </c>
+      <c r="B23" t="s">
+        <v>115</v>
+      </c>
+      <c r="C23" t="s">
+        <v>118</v>
+      </c>
+      <c r="D23" t="s">
+        <v>120</v>
+      </c>
+      <c r="E23" t="s">
+        <v>119</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23" t="s">
+        <v>44</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+      <c r="M23" t="s">
+        <v>121</v>
+      </c>
+      <c r="N23" t="s">
+        <v>122</v>
+      </c>
+      <c r="O23">
+        <v>0</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>118</v>
+      </c>
+      <c r="T23">
+        <v>1</v>
+      </c>
+      <c r="U23">
+        <v>-180</v>
+      </c>
+      <c r="V23">
+        <v>180</v>
+      </c>
+      <c r="W23">
+        <v>0</v>
+      </c>
+      <c r="X23">
+        <v>0</v>
+      </c>
+      <c r="AA23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>125</v>
+      </c>
+      <c r="B24" t="s">
+        <v>125</v>
+      </c>
+      <c r="C24" t="s">
+        <v>123</v>
+      </c>
+      <c r="D24" t="s">
+        <v>143</v>
+      </c>
+      <c r="E24" t="s">
+        <v>124</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24" t="s">
+        <v>31</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+      <c r="M24" t="s">
+        <v>126</v>
+      </c>
+      <c r="N24" t="s">
+        <v>127</v>
+      </c>
+      <c r="O24">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>123</v>
+      </c>
+      <c r="T24">
+        <v>1</v>
+      </c>
+      <c r="U24">
+        <v>5</v>
+      </c>
+      <c r="V24">
+        <v>180</v>
+      </c>
+      <c r="W24">
+        <v>3</v>
+      </c>
+      <c r="X24">
+        <v>1</v>
+      </c>
+      <c r="Y24">
+        <v>1</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>125</v>
+      </c>
+      <c r="B25" t="s">
+        <v>125</v>
+      </c>
+      <c r="C25" t="s">
+        <v>128</v>
+      </c>
+      <c r="D25" t="s">
+        <v>144</v>
+      </c>
+      <c r="E25" t="s">
+        <v>129</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25" t="s">
+        <v>27</v>
+      </c>
+      <c r="K25">
+        <v>1</v>
+      </c>
+      <c r="O25">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>128</v>
+      </c>
+      <c r="T25">
+        <v>0</v>
+      </c>
+      <c r="W25">
+        <v>0</v>
+      </c>
+      <c r="X25">
+        <v>0</v>
+      </c>
+      <c r="AA25">
         <v>0</v>
       </c>
     </row>

</xml_diff>